<commit_message>
MAJ des modèles métier+Mapping(Img,LabReport) 448ea0207b1c8f3a572f9526cfbec3f5fe2226c9
</commit_message>
<xml_diff>
--- a/update-ml-labreport-laboratoryobservation/ig/FRSectionImagingSupportingInformationLMCDAFHIR.xlsx
+++ b/update-ml-labreport-laboratoryobservation/ig/FRSectionImagingSupportingInformationLMCDAFHIR.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="70">
   <si>
     <t>Property</t>
   </si>
@@ -62,7 +62,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-14T13:28:49+00:00</t>
+    <t>2026-09-16T13:00:57+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -86,7 +86,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Mapping des éléments du modèle métier FRLMImagingSupportingInformation vers la section CDA FRCDADICOMHistoriqueMedical, puis vers la section FHIR FRCompositionDocument.section:sectionHistory et le profil FRDiagnosticReportImagingDocument.</t>
+    <t>Mapping des éléments du modèle métier FRLMSupportingInformation (partagé avec le mapping biologie) vers la section CDA FRCDADICOMHistoriqueMedical, puis vers la section FHIR FRCompositionDocument.section:sectionHistory et le profil FRDiagnosticReportImagingDocument, pour le contexte imagerie.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -107,7 +107,7 @@
     <t>Target</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/document-core/StructureDefinition/FRLMImagingSupportingInformation|0.1.0</t>
+    <t>https://interop.esante.gouv.fr/ig/document-core/StructureDefinition/FRLMSupportingInformation|0.1.0</t>
   </si>
   <si>
     <t/>
@@ -116,7 +116,7 @@
     <t>https://interop.esante.gouv.fr/ig/cda/document-core/StructureDefinition/fr-cda-dicom-historique-medical|0.1.0</t>
   </si>
   <si>
-    <t>FRLMImagingSupportingInformation</t>
+    <t>FRLMSupportingInformation</t>
   </si>
   <si>
     <t>equivalent</t>
@@ -128,46 +128,34 @@
     <t>FRCDADICOMHistoriqueMedical</t>
   </si>
   <si>
-    <t>FRLMImagingSupportingInformation.codeSection</t>
+    <t>FRLMSupportingInformation.codeSection</t>
   </si>
   <si>
     <t>Section.code</t>
   </si>
   <si>
-    <t>FRLMImagingSupportingInformation.titleSection</t>
+    <t>FRLMSupportingInformation.titleSection</t>
   </si>
   <si>
     <t>Section.title</t>
   </si>
   <si>
-    <t>FRLMImagingSupportingInformation.description</t>
+    <t>FRLMSupportingInformation.description</t>
   </si>
   <si>
     <t>Section.text</t>
   </si>
   <si>
-    <t>FRLMImagingSupportingInformation.entry.historyOfPastIllness</t>
+    <t>FRLMSupportingInformation.entry.observation</t>
   </si>
   <si>
     <t>FRLMObservation</t>
   </si>
   <si>
-    <t>Section.entry.observation</t>
-  </si>
-  <si>
-    <t>FRCDASimpleObservation</t>
-  </si>
-  <si>
-    <t>FRLMImagingSupportingInformation.entry.historyOfPastProcedures</t>
-  </si>
-  <si>
-    <t>FRLMImagingSupportingInformation.entry.pregnancyStatus</t>
-  </si>
-  <si>
-    <t>FRCDAObservationSurLaGrossesse</t>
-  </si>
-  <si>
-    <t>FRLMImagingSupportingInformation.entry.contraIndication</t>
+    <t>Section.section.entry.observation</t>
+  </si>
+  <si>
+    <t>FRCDASectionDICOMHistoriqueMedical.entry(FRCDASimpleObservation)</t>
   </si>
   <si>
     <t>https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-composition-document|0.1.0</t>
@@ -188,30 +176,42 @@
     <t>Composition.section.text</t>
   </si>
   <si>
-    <t>FRLMImagingSupportingInformation.entry.previousResultsInformation</t>
-  </si>
-  <si>
     <t>Composition.section.entry</t>
   </si>
   <si>
     <t>Observation</t>
   </si>
   <si>
+    <t>FRLMSupportingInformation.entry.condition</t>
+  </si>
+  <si>
     <t>FRLMCondition</t>
   </si>
   <si>
     <t>FRConditionDocument</t>
   </si>
   <si>
-    <t>FRObservationContraIndicationsDocument</t>
-  </si>
-  <si>
-    <t>FRLMImagingSupportingInformation.entry.condition</t>
+    <t>FRLMSupportingInformation.entry.device</t>
+  </si>
+  <si>
+    <t>FRDeviceUseStatementDocument</t>
+  </si>
+  <si>
+    <t>FRLMSupportingInformation.entry.pregnancyStatus</t>
   </si>
   <si>
     <t>FRObservationPregnancyDocument</t>
   </si>
   <si>
+    <t>FRLMSupportingInformation.entry.medicationAdministration</t>
+  </si>
+  <si>
+    <t>FRLMDICOMMedicationAdministration</t>
+  </si>
+  <si>
+    <t>FRMedicationAdministrationDocument</t>
+  </si>
+  <si>
     <t>https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-diagnostic-report-imaging-document|0.1.0</t>
   </si>
   <si>
@@ -221,13 +221,10 @@
     <t>FRDiagnosticReportImagingDocument.extension:historiqueMedical</t>
   </si>
   <si>
-    <t>DiagnosticReport.result:resultatAnterieur</t>
-  </si>
-  <si>
-    <t>FRLMImagingSupportingInformation.entry.device</t>
-  </si>
-  <si>
-    <t>FRLMImagingSupportingInformation.entry.priorMedicationAdministration</t>
+    <t>Observation or FRObservationPregnancyDocument or FRObservationContraIndicationsImagingDocument</t>
+  </si>
+  <si>
+    <t>Device</t>
   </si>
 </sst>
 </file>
@@ -483,7 +480,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -588,51 +585,6 @@
         <v>45</v>
       </c>
       <c r="E7" t="s" s="2">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="2">
-        <v>47</v>
-      </c>
-      <c r="B8" s="2"/>
-      <c r="C8" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s" s="2">
-        <v>45</v>
-      </c>
-      <c r="E8" t="s" s="2">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="2">
-        <v>48</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D9" t="s" s="2">
-        <v>45</v>
-      </c>
-      <c r="E9" t="s" s="2">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="2">
-        <v>50</v>
-      </c>
-      <c r="B10" s="2"/>
-      <c r="C10" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D10" t="s" s="2">
-        <v>45</v>
-      </c>
-      <c r="E10" t="s" s="2">
         <v>46</v>
       </c>
     </row>
@@ -643,7 +595,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -674,7 +626,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -689,10 +641,10 @@
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
@@ -704,7 +656,7 @@
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E4" s="2"/>
     </row>
@@ -717,7 +669,7 @@
         <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E5" s="2"/>
     </row>
@@ -730,116 +682,88 @@
         <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>57</v>
-      </c>
-      <c r="B7" s="2"/>
+        <v>43</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>44</v>
+      </c>
       <c r="C7" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s" s="2">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s" s="2">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>43</v>
-      </c>
-      <c r="B9" t="s" s="2">
-        <v>60</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E9" t="s" s="2">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E10" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>50</v>
-      </c>
-      <c r="B11" s="2"/>
+        <v>62</v>
+      </c>
+      <c r="B11" t="s" s="2">
+        <v>63</v>
+      </c>
       <c r="C11" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E11" t="s" s="2">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="2">
-        <v>63</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D12" t="s" s="2">
-        <v>58</v>
-      </c>
-      <c r="E12" t="s" s="2">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="2">
-        <v>48</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D13" t="s" s="2">
-        <v>58</v>
-      </c>
-      <c r="E13" t="s" s="2">
         <v>64</v>
       </c>
     </row>
@@ -850,7 +774,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -904,20 +828,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
+        <v>66</v>
+      </c>
+      <c r="E4" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="E4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" t="s" s="2">
@@ -926,11 +852,13 @@
       <c r="D5" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="E5" s="2"/>
+      <c r="E5" t="s" s="2">
+        <v>57</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" t="s" s="2">
@@ -939,72 +867,26 @@
       <c r="D6" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="E6" s="2"/>
+      <c r="E6" t="s" s="2">
+        <v>69</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>50</v>
-      </c>
-      <c r="B7" s="2"/>
+        <v>62</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>63</v>
+      </c>
       <c r="C7" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="2">
-        <v>63</v>
-      </c>
-      <c r="B8" s="2"/>
-      <c r="C8" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s" s="2">
-        <v>66</v>
-      </c>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="2">
-        <v>69</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D9" t="s" s="2">
-        <v>66</v>
-      </c>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="2">
-        <v>48</v>
-      </c>
-      <c r="B10" s="2"/>
-      <c r="C10" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D10" t="s" s="2">
-        <v>66</v>
-      </c>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="2">
-        <v>70</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D11" t="s" s="2">
-        <v>66</v>
-      </c>
-      <c r="E11" s="2"/>
+      <c r="E7" t="s" s="2">
+        <v>64</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>